<commit_message>
Fix bid line import validation defaults
</commit_message>
<xml_diff>
--- a/public/templates/zla-bid-line-import-template.xlsx
+++ b/public/templates/zla-bid-line-import-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Re28f78a78b76495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bid Lines" sheetId="2" r:id="R6927270acb8e4f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R9df71cd8f7db4985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rb78092b80eca4efb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R71fe18df3f544edf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bid Lines" sheetId="2" r:id="R37cf2db8df664f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R8447305ceca94ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rb9a00dd486984ecf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -353,7 +353,7 @@
         <x:color rgb="FF8B2D28"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E5"/>
         </x:patternFill>
       </x:fill>
@@ -649,7 +649,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Use the dropdown values for Type, Fatigue Group, Mid, AWS, 4/10, and Flex.</x:v>
+        <x:v>Use the dropdowns when needed. Fatigue Group, AWS, and Flex may be left blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -697,7 +697,7 @@
         <x:v>fatigue_group</x:v>
       </x:c>
       <x:c r="B16" s="26" t="str">
-        <x:v>A, B, C, or C only. Blank values default to C.</x:v>
+        <x:v>Optional. A, B, C, or C only. Blank keeps the current value when updating and defaults to C for a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
@@ -713,7 +713,7 @@
         <x:v>aws</x:v>
       </x:c>
       <x:c r="B18" s="26" t="str">
-        <x:v>Yes or No.</x:v>
+        <x:v>Optional. Yes or No. Blank keeps the current value when updating and defaults to No for a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
@@ -729,7 +729,7 @@
         <x:v>flex</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Yes or No.</x:v>
+        <x:v>Optional. Yes or No. Blank keeps the current value when updating and defaults to Yes for a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -737,7 +737,7 @@
         <x:v>Sunday-Saturday</x:v>
       </x:c>
       <x:c r="B21" s="26" t="str">
-        <x:v>Required. A shift code or RDO in every day column.</x:v>
+        <x:v>Required. Enter a shift code or RDO in every day column. RDO, R.D.O., and similar punctuation are accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -2548,7 +2548,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24a625232a644238"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdce1e3dc754549"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2631,21 +2631,15 @@
       <x:c r="C2" s="58" t="str">
         <x:v>F/S</x:v>
       </x:c>
-      <x:c r="D2" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
+      <x:c r="D2" s="58"/>
       <x:c r="E2" s="58" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="F2" s="58" t="str">
-        <x:v>No</x:v>
-      </x:c>
+      <x:c r="F2" s="58"/>
       <x:c r="G2" s="58" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="H2" s="58" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
+      <x:c r="H2" s="58"/>
       <x:c r="I2" s="58" t="str">
         <x:v>700</x:v>
       </x:c>
@@ -2766,10 +2760,10 @@
         <x:v>fatigue_group</x:v>
       </x:c>
       <x:c r="B5" s="63" t="str">
-        <x:v>A, B, C, C only</x:v>
+        <x:v>Optional: A, B, C, C only</x:v>
       </x:c>
       <x:c r="C5" s="64" t="str">
-        <x:v>Use the published fatigue classification.</x:v>
+        <x:v>Blank preserves an existing value or defaults to C on a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2788,10 +2782,10 @@
         <x:v>aws</x:v>
       </x:c>
       <x:c r="B7" s="63" t="str">
-        <x:v>No, Yes</x:v>
+        <x:v>Optional: No, Yes</x:v>
       </x:c>
       <x:c r="C7" s="64" t="str">
-        <x:v>Alternative work schedule indicator.</x:v>
+        <x:v>Blank preserves an existing value or defaults to No on a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2810,10 +2804,10 @@
         <x:v>flex</x:v>
       </x:c>
       <x:c r="B9" s="63" t="str">
-        <x:v>No, Yes</x:v>
+        <x:v>Optional: No, Yes</x:v>
       </x:c>
       <x:c r="C9" s="64" t="str">
-        <x:v>Flex line indicator.</x:v>
+        <x:v>Blank preserves an existing value or defaults to Yes on a new line.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2824,7 +2818,7 @@
         <x:v>Shift code or RDO</x:v>
       </x:c>
       <x:c r="C10" s="66" t="str">
-        <x:v>All seven day cells are required.</x:v>
+        <x:v>All seven day cells are required. RDO, R.D.O., and similar punctuation are accepted.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>